<commit_message>
Add 2phase Clock Circuit.
Add 2phase Clock Circuit.
</commit_message>
<xml_diff>
--- a/docs/pin_list.xlsx
+++ b/docs/pin_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b2da16fa1785921/MyDocuments/Community/ISHIKAI/shuttle/OpenSUSI-TR10/2026/KOSEN/KOSENKIKO/OpenSUSI-TR1um-v2609_01/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="342" documentId="11_AD4D066CA252ABDACC1048686197E6B673EEDF5D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80117ADE-0D64-4D1C-9914-8DC132CAB8C3}"/>
+  <xr:revisionPtr revIDLastSave="350" documentId="11_AD4D066CA252ABDACC1048686197E6B673EEDF5D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2647B63-341A-4259-B637-403F22146109}"/>
   <bookViews>
     <workbookView xWindow="38330" yWindow="0" windowWidth="19200" windowHeight="9980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
   <si>
     <t>Pin Number</t>
     <phoneticPr fontId="1"/>
@@ -86,10 +86,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>none</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>IN</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -99,6 +95,26 @@
   </si>
   <si>
     <t>inverter</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2phase_CLK</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VDD</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CLK</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PH1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>PH2</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -232,6 +248,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -567,28 +587,32 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7" spans="1:3" ht="18.350000000000001" thickBot="1">
       <c r="A7" s="5">
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="6"/>
+        <v>17</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8" spans="1:3" ht="18.350000000000001" thickTop="1">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -607,10 +631,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="18.350000000000001" thickBot="1">
@@ -618,7 +642,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>2</v>
@@ -629,18 +653,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="9"/>
+        <v>17</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="2"/>
+        <v>17</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1">

</xml_diff>